<commit_message>
Update reports 2026-10-26 10:06
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-26.xlsx
+++ b/gex_pivot_levels_2026-10-26.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -610,12 +610,12 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>+$1.04M</t>
+          <t>+$825.87K</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>+$4.73M</t>
+          <t>+$3.75M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -643,12 +643,12 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>-$12.25M</t>
+          <t>-$10.09M</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>+$12.83M</t>
+          <t>+$10.56M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -709,12 +709,12 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>-$7.06M</t>
+          <t>-$5.98M</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>+$7.42M</t>
+          <t>+$6.28M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -738,12 +738,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>-$4.43M</t>
+          <t>-$3.87M</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>+$5.09M</t>
+          <t>+$4.45M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -767,12 +767,12 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>-$1.85M</t>
+          <t>-$1.64M</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>+$2.66M</t>
+          <t>+$2.34M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>-$8.25M</t>
+          <t>-$7.20M</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>+$12.46M</t>
+          <t>+$10.87M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -833,12 +833,12 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>-$3.39M</t>
+          <t>-$3.25M</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>+$20.49M</t>
+          <t>+$19.60M</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>-$1.46M</t>
+          <t>-$1.52M</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>+$20.62M</t>
+          <t>+$21.46M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -986,12 +986,12 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>+$8.00M</t>
+          <t>+$8.81M</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>+$18.18M</t>
+          <t>+$19.99M</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>-$395.21K</t>
+          <t>-$450.79K</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>+$8.13M</t>
+          <t>+$9.28M</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>+$2.10M</t>
+          <t>+$2.45M</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>+$8.41M</t>
+          <t>+$9.81M</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1101,58 +1101,58 @@
       <c r="G19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>7731.49</v>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>766</v>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>-$51.35M</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>+$62.12M</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A20" s="5" t="n">
+        <v>7727.32</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>7680</v>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>+$4.24M</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>+$8.00M</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>7737.32</v>
+        <v>7731.49</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>7690</v>
+        <v>766</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>+$5.04M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>-$51.35M</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>+$8.69M</t>
+          <t>+$62.12M</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1162,70 +1162,173 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
+        <v>7732.32</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>7685</v>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>+$734.77K</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>+$7.90M</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>7737.32</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>7690</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>+$6.27M</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>+$10.81M</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
         <v>7747.32</v>
       </c>
-      <c r="B22" s="5" t="n">
+      <c r="B24" s="2" t="n">
         <v>7700</v>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>-$258.82K</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>+$18.36M</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>-$340.17K</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>+$24.13M</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>7772.32</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7725</v>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>+$2.43M</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>+$6.62M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="n">
-        <v>7772.32</v>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>7725</v>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>7777.32</v>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>7730</v>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>+$1.77M</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>+$4.82M</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr"/>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>+$3.44M</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>+$4.88M</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G23"/>
+  <autoFilter ref="A1:G26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2699,7 +2802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2945,38 +3048,42 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>7697.32</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>7650</v>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="B7" s="2" t="n">
+        <v>7747.32</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>7700</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>-$1.46M</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>+$20.62M</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>-$340.17K</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>+$24.13M</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2985,130 +3092,130 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
+        <v>7697.32</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>7650</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>-$1.52M</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>+$21.46M</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>7707.32</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>7660</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>+$8.81M</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>+$19.99M</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
         <v>7672.32</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C10" s="5" t="n">
         <v>7625</v>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>-$3.39M</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>+$20.49M</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>-$3.25M</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>+$19.60M</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>7747.32</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>7700</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>-$258.82K</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>+$18.36M</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>28723.82</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>695</v>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>-$18.06M</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>+$18.20M</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>7707.32</v>
+        <v>28723.82</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7660</v>
+        <v>695</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>+$8.00M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>-$18.06M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>+$18.18M</t>
+          <t>+$18.20M</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -3118,7 +3225,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3167,10 +3274,10 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>7612.32</v>
+        <v>7647.32</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>7565</v>
+        <v>7600</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
@@ -3179,12 +3286,12 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>-$12.25M</t>
+          <t>-$7.20M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>+$12.83M</t>
+          <t>+$10.87M</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -3205,24 +3312,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>7647.32</v>
+        <v>7737.32</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>7600</v>
+        <v>7690</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>-$8.25M</t>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>+$6.27M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>+$12.46M</t>
+          <t>+$10.81M</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -3232,7 +3339,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -3277,112 +3384,112 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>7612.32</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>7565</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>-$10.09M</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>+$10.56M</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>29340.46</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C17" s="2" t="n">
         <v>710</v>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>-$2.58M</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>+$10.24M</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
-        <v>7687.32</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>7640</v>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="B18" s="5" t="n">
+        <v>7722.32</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>7675</v>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>-$1.37M</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>+$9.20M</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>+$2.45M</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>+$9.81M</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>7737.32</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>7690</v>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>+$5.04M</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>+$8.69M</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -3391,32 +3498,36 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>7722.32</v>
+        <v>7717.32</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>7675</v>
+        <v>7670</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>+$2.10M</t>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>-$450.79K</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>+$8.41M</t>
+          <t>+$9.28M</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -3425,10 +3536,10 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>7717.32</v>
+        <v>7687.32</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>7670</v>
+        <v>7640</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
@@ -3437,24 +3548,20 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>-$395.21K</t>
+          <t>-$1.37M</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>+$8.13M</t>
+          <t>+$9.20M</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -3463,24 +3570,24 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>7681.33</v>
+        <v>7727.32</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>761</v>
+        <v>7680</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>-$4.19M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>+$4.24M</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>+$7.96M</t>
+          <t>+$8.00M</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -3501,362 +3608,370 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
+        <v>7681.33</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>761</v>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>-$4.19M</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>+$7.96M</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>7732.32</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>7685</v>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>+$734.77K</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>+$7.90M</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>2846.98</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>283</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>+$7.41M</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>+$7.41M</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7772.32</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>7725</v>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>+$2.43M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>+$6.62M</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2756.44</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>274</v>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>-$2.55M</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>+$6.45M</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
         <v>7622.32</v>
       </c>
-      <c r="C22" s="5" t="n">
+      <c r="C27" s="5" t="n">
         <v>7575</v>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>-$7.06M</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>+$7.42M</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>-$5.98M</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>+$6.28M</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
-        <v>2846.98</v>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>283</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="B28" s="2" t="n">
+        <v>2816.8</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>+$7.41M</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>+$7.41M</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>+$5.82M</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>+$6.21M</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>2756.44</v>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>274</v>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>-$2.55M</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>+$6.45M</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>29546.01</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>715</v>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>+$1.23M</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>+$5.88M</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>4058.79</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>370</v>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>-$2.40M</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>+$5.69M</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>2816.8</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>280</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>+$5.82M</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>+$6.21M</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>29546.01</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>715</v>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="inlineStr">
-        <is>
-          <t>+$1.23M</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>+$5.88M</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>4058.79</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>370</v>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>-$2.40M</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>+$5.69M</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>2746.38</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>273</v>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>+$1.32M</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>+$5.54M</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="n">
-        <v>29751.56</v>
-      </c>
-      <c r="C29" s="5" t="n">
-        <v>720</v>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>-$1.14M</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>+$5.39M</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>29134.91</v>
-      </c>
-      <c r="C30" s="5" t="n">
-        <v>705</v>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>-$1.99M</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>+$5.17M</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>7637.32</v>
+        <v>2746.38</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>7590</v>
+        <v>273</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>-$4.43M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>+$1.32M</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>+$5.09M</t>
+          <t>+$5.54M</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -3865,24 +3980,24 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>29422.68</v>
+        <v>29751.56</v>
       </c>
       <c r="C32" s="5" t="n">
-        <v>712</v>
+        <v>720</v>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>+$429.31K</t>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>-$1.14M</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>+$5.06M</t>
+          <t>+$5.39M</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -3895,28 +4010,28 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>7772.32</v>
+        <v>29134.91</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>7725</v>
+        <v>705</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>+$1.77M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>-$1.99M</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>+$4.82M</t>
+          <t>+$5.17M</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -3929,66 +4044,62 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>7602.32</v>
+        <v>29422.68</v>
       </c>
       <c r="C34" s="5" t="n">
-        <v>7555</v>
+        <v>712</v>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>+$1.04M</t>
+          <t>+$429.31K</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>+$4.73M</t>
+          <t>+$5.06M</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>29093.81</v>
+        <v>7777.32</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>704</v>
+        <v>7730</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>+$1.02M</t>
+          <t>+$3.44M</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>+$3.67M</t>
+          <t>+$4.88M</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -4005,40 +4116,36 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>2706.14</v>
+        <v>7637.32</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>269</v>
+        <v>7590</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>IWM</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>-$3.29M</t>
+          <t>-$3.87M</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>+$3.57M</t>
+          <t>+$4.45M</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H36" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -4047,24 +4154,24 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>7581.02</v>
+        <v>7602.32</v>
       </c>
       <c r="C37" s="5" t="n">
-        <v>751</v>
+        <v>7555</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>-$2.96M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>+$825.87K</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>+$3.01M</t>
+          <t>+$3.75M</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
@@ -4079,38 +4186,38 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n">
-        <v>98.26000000000001</v>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>165</v>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
-        <is>
-          <t>+$2.98M</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>+$2.98M</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>29093.81</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>704</v>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>+$1.02M</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>+$3.67M</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4123,24 +4230,24 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>2806.74</v>
+        <v>2706.14</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>+$633.43K</t>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>-$3.29M</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>+$2.88M</t>
+          <t>+$3.57M</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
@@ -4161,24 +4268,24 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>7642.32</v>
+        <v>7581.02</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>7595</v>
+        <v>751</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>-$1.85M</t>
+          <t>-$2.96M</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>+$2.66M</t>
+          <t>+$3.01M</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -4195,28 +4302,28 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>4061.72</v>
+        <v>98.26000000000001</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>81</v>
+        <v>165</v>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>-$1.30M</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>+$2.98M</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>+$1.43M</t>
+          <t>+$2.98M</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -4226,7 +4333,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4237,10 +4344,10 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>2836.92</v>
+        <v>2806.74</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
@@ -4249,12 +4356,12 @@
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>+$1.26M</t>
+          <t>+$633.43K</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>+$1.33M</t>
+          <t>+$2.88M</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -4269,40 +4376,40 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="n">
-        <v>92.31</v>
-      </c>
-      <c r="C43" s="2" t="n">
-        <v>155</v>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>-$1.20M</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>+$1.24M</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>7642.32</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>7595</v>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>-$1.64M</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>+$2.34M</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4313,10 +4420,10 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>4162.01</v>
+        <v>4061.72</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
@@ -4325,12 +4432,12 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>-$1.06M</t>
+          <t>-$1.30M</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>+$1.19M</t>
+          <t>+$1.43M</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -4347,62 +4454,66 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>104.22</v>
+        <v>2836.92</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>175</v>
+        <v>282</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>+$302.57K</t>
+          <t>+$1.26M</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>+$302.57K</t>
+          <t>+$1.33M</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>29112.72</v>
+        <v>92.31</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>28960</v>
+        <v>155</v>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E46" s="9" t="inlineStr">
-        <is>
-          <t>+$145.95K</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>-$1.20M</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>+$229.34K</t>
+          <t>+$1.24M</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -4412,81 +4523,81 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="n">
-        <v>29152.72</v>
-      </c>
-      <c r="C47" s="5" t="n">
-        <v>29000</v>
-      </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>-$4.63K</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>+$199.23K</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>4162.01</v>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>-$1.06M</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>+$1.19M</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>104.22</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>+$302.57K</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>+$302.57K</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H47" s="6" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>29072.72</v>
-      </c>
-      <c r="C48" s="2" t="n">
-        <v>28920</v>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>-$129.73K</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>+$139.00K</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H48" s="6" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -4495,24 +4606,24 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>29082.72</v>
+        <v>29112.72</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>28930</v>
+        <v>28960</v>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>-$136.68K</t>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>+$145.95K</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>+$136.68K</t>
+          <t>+$229.34K</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -4522,81 +4633,81 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>4111.86</v>
+        <v>29152.72</v>
       </c>
       <c r="C50" s="5" t="n">
-        <v>82</v>
+        <v>29000</v>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>-$132</t>
+          <t>-$4.63K</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>+$117.20K</t>
+          <t>+$199.23K</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B51" s="5" t="n">
-        <v>29052.72</v>
-      </c>
-      <c r="C51" s="5" t="n">
-        <v>28900</v>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="B51" s="2" t="n">
+        <v>29072.72</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>28920</v>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>-$97.30K</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>+$111.20K</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="inlineStr"/>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>-$129.73K</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>+$139.00K</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -4605,24 +4716,24 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>29182.72</v>
+        <v>29082.72</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>29030</v>
+        <v>28930</v>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E52" s="9" t="inlineStr">
-        <is>
-          <t>+$69.50K</t>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>-$136.68K</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>+$92.66K</t>
+          <t>+$136.68K</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -4632,115 +4743,119 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>4111.86</v>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>-$132</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>+$117.20K</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B53" s="5" t="n">
-        <v>29252.72</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>29100</v>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="B54" s="5" t="n">
+        <v>29052.72</v>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>28900</v>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>+$6.95K</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>+$67.18K</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>-$97.30K</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>+$111.20K</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="H54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B54" s="2" t="n">
-        <v>29002.72</v>
-      </c>
-      <c r="C54" s="2" t="n">
-        <v>28850</v>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="B55" s="2" t="n">
+        <v>29182.72</v>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>29030</v>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>-$50.97K</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>+$60.23K</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="n">
-        <v>29202.72</v>
-      </c>
-      <c r="C55" s="5" t="n">
-        <v>29050</v>
-      </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>+$2.32K</t>
-        </is>
-      </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>+$57.92K</t>
-        </is>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H55" s="6" t="inlineStr"/>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>+$69.50K</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>+$92.66K</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -4749,10 +4864,10 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>29302.72</v>
+        <v>29252.72</v>
       </c>
       <c r="C56" s="5" t="n">
-        <v>29150</v>
+        <v>29100</v>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
@@ -4761,12 +4876,12 @@
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>+$44.02K</t>
+          <t>+$6.95K</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>+$57.92K</t>
+          <t>+$67.18K</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
@@ -4783,10 +4898,10 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>29172.72</v>
+        <v>29002.72</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>29020</v>
+        <v>28850</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
@@ -4795,12 +4910,12 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>-$16.22K</t>
+          <t>-$50.97K</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>+$39.38K</t>
+          <t>+$60.23K</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -4821,24 +4936,24 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>28952.72</v>
+        <v>29202.72</v>
       </c>
       <c r="C58" s="5" t="n">
-        <v>28800</v>
+        <v>29050</v>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E58" s="7" t="inlineStr">
-        <is>
-          <t>-$28.38K</t>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>+$2.32K</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>+$32.43K</t>
+          <t>+$57.92K</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -4855,72 +4970,68 @@
         </is>
       </c>
       <c r="B59" s="5" t="n">
-        <v>29077.72</v>
+        <v>29302.72</v>
       </c>
       <c r="C59" s="5" t="n">
-        <v>28925</v>
+        <v>29150</v>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr">
-        <is>
-          <t>-$23.17K</t>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>+$44.02K</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>+$23.17K</t>
+          <t>+$57.92K</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H59" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B60" s="5" t="n">
-        <v>29012.72</v>
-      </c>
-      <c r="C60" s="5" t="n">
-        <v>28860</v>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
+      <c r="B60" s="2" t="n">
+        <v>29172.72</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>29020</v>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>+$2.32K</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>+$20.85K</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>-$16.22K</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>+$39.38K</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4931,39 +5042,149 @@
         </is>
       </c>
       <c r="B61" s="5" t="n">
+        <v>28952.72</v>
+      </c>
+      <c r="C61" s="5" t="n">
+        <v>28800</v>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>-$28.38K</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>+$32.43K</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="n">
+        <v>29077.72</v>
+      </c>
+      <c r="C62" s="5" t="n">
+        <v>28925</v>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>-$23.17K</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>+$23.17K</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>29012.72</v>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>28860</v>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>+$2.32K</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>+$20.85K</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="n">
         <v>29292.72</v>
       </c>
-      <c r="C61" s="5" t="n">
+      <c r="C64" s="5" t="n">
         <v>29140</v>
       </c>
-      <c r="D61" s="6" t="inlineStr">
+      <c r="D64" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E61" s="7" t="inlineStr">
+      <c r="E64" s="7" t="inlineStr">
         <is>
           <t>-$20.85K</t>
         </is>
       </c>
-      <c r="F61" s="6" t="inlineStr">
+      <c r="F64" s="6" t="inlineStr">
         <is>
           <t>+$20.85K</t>
         </is>
       </c>
-      <c r="G61" s="6" t="inlineStr">
+      <c r="G64" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H61" s="6" t="inlineStr">
+      <c r="H64" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H61"/>
+  <autoFilter ref="A1:H64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>